<commit_message>
Mô tả thay đổi
</commit_message>
<xml_diff>
--- a/public/MAU_IMPORT_NHAN_VIEN.xlsx
+++ b/public/MAU_IMPORT_NHAN_VIEN.xlsx
@@ -402,11 +402,12 @@
             <sz val="10"/>
             <rFont val="Times New Roman"/>
           </rPr>
-          <t xml:space="preserve">• Nhập 1; 2; 3 (tách bằng dấu ;), hoặc để trống.
+          <t xml:space="preserve">• Nhập 1; 2; 3; 4 (tách bằng dấu ;), hoặc để trống.
 • Ví dụ: 1; 3.
 1: lớp có % áp dụng 80%.
 2: chỉ Lớp kèm ONL áp dụng 80%.
-3: IELTS - 56% ONL áp dụng 100%. Ưu tiên 3 → 2 → 1; không giảm hai lần.</t>
+3: IELTS - 56% ONL áp dụng 100%. 4: Lớp chung có % dùng 170.000đ/giờ. Ưu tiên 4 → 3 → 2/1.
+• Không giảm thêm 20%.</t>
         </r>
       </text>
     </comment>
@@ -882,11 +883,12 @@
             <sz val="10"/>
             <rFont val="Times New Roman"/>
           </rPr>
-          <t xml:space="preserve">• Nhập 1; 2; 3 (tách bằng dấu ;), hoặc để trống.
+          <t xml:space="preserve">• Nhập 1; 2; 3; 4 (tách bằng dấu ;), hoặc để trống.
 • Ví dụ: 1; 3.
 1: lớp có % áp dụng 80%.
 2: chỉ Lớp kèm ONL áp dụng 80%.
-3: IELTS - 56% ONL áp dụng 100%. Ưu tiên 3 → 2 → 1; không giảm hai lần.</t>
+3: IELTS - 56% ONL áp dụng 100%. 4: Lớp chung có % dùng 170.000đ/giờ. Ưu tiên 4 → 3 → 2/1.
+• Không giảm thêm 20%.</t>
         </r>
       </text>
     </comment>
@@ -1362,11 +1364,12 @@
             <sz val="10"/>
             <rFont val="Times New Roman"/>
           </rPr>
-          <t xml:space="preserve">• Nhập 1; 2; 3 (tách bằng dấu ;), hoặc để trống.
+          <t xml:space="preserve">• Nhập 1; 2; 3; 4 (tách bằng dấu ;), hoặc để trống.
 • Ví dụ: 1; 3.
 1: lớp có % áp dụng 80%.
 2: chỉ Lớp kèm ONL áp dụng 80%.
-3: IELTS - 56% ONL áp dụng 100%. Ưu tiên 3 → 2 → 1; không giảm hai lần.</t>
+3: IELTS - 56% ONL áp dụng 100%. 4: Lớp chung có % dùng 170.000đ/giờ. Ưu tiên 4 → 3 → 2/1.
+• Không giảm thêm 20%.</t>
         </r>
       </text>
     </comment>
@@ -2288,7 +2291,7 @@
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Không cần chấm công" prompt="1 = Không cần chấm công; 0/trống = không bật." sqref="Q2:Q1000">
       <formula1>TRUE</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Cơ chế lương đặc biệt" prompt="Nhập 1; 2; 3 (tách bằng dấu ;), hoặc để trống. Ví dụ: 1; 3. 1: lớp có % áp dụng 80%. 2: chỉ Lớp kèm ONL áp dụng 80%. 3: IELTS - 56% ONL áp dụng 100%. Ưu tiên 3 → 2 → 1; không giảm hai lần." sqref="R2:R1000">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Cơ chế lương đặc biệt" prompt="Nhập 1; 2; 3; 4 (tách bằng dấu ;), hoặc để trống. Ví dụ: 1; 3. 1: lớp có % áp dụng 80%. 2: chỉ Lớp kèm ONL áp dụng 80%. 3: IELTS - 56% ONL áp dụng 100%. 4: Lớp chung có % dùng 170.000đ/giờ. Ưu tiên 4 → 3 → 2/1. Không giảm thêm 20%." sqref="R2:R1000">
       <formula1>TRUE</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Email" prompt="Email của nhân viên. Có thể để trống." sqref="S2:S1000">

</xml_diff>